<commit_message>
Data Driven Testing - Sending Data To Application
</commit_message>
<xml_diff>
--- a/selenium-maven-project/TestData/caldata.xlsx
+++ b/selenium-maven-project/TestData/caldata.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="15">
   <si>
     <t>Principle</t>
   </si>
@@ -155,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -171,6 +171,21 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="true"/>
@@ -553,7 +568,7 @@
       <c r="G2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="H2" t="s" s="12">
+      <c r="H2" t="s" s="27">
         <v>14</v>
       </c>
     </row>
@@ -579,7 +594,7 @@
       <c r="G3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="H3" t="s" s="13">
+      <c r="H3" t="s" s="28">
         <v>14</v>
       </c>
     </row>
@@ -605,7 +620,7 @@
       <c r="G4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="H4" t="s" s="14">
+      <c r="H4" t="s" s="29">
         <v>14</v>
       </c>
     </row>
@@ -631,7 +646,7 @@
       <c r="G5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="H5" t="s" s="15">
+      <c r="H5" t="s" s="30">
         <v>14</v>
       </c>
     </row>
@@ -657,7 +672,7 @@
       <c r="G6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H6" t="s" s="16">
+      <c r="H6" t="s" s="31">
         <v>13</v>
       </c>
     </row>

</xml_diff>